<commit_message>
Verify Payment Analytics cases against QA: 91 of 149 now confirmed
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -1470,7 +1470,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised in this run - only the 12-month path was driven.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: selecting Last 3 Months redrew the chart with exactly 3 month labels.</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised in this run.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: selecting Last 24 Months redrew the chart with exactly 24 month labels spanning two years.</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2173,7 @@
       <c r="N21" s="2"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Paymentus account exists in credentials/qa.json - cannot be run on QA today.</t>
+          <t xml:space="preserve">QA 2026-09-15 Paymentus: legend read ['Ach','Token','Card'] - the only gateway showing all three series.</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2562,7 @@
       <c r="N25" s="2"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Paymentus account available.</t>
+          <t xml:space="preserve">QA 2026-09-15 Paymentus: tooltip showed Ach(29), Token(246) and Card(63) together.</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       <c r="N26" s="2"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - hover tooltip not driven in this run.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: tooltip read Token(3) and Card(52); the summary cards for the same month read Token (3) and Card (52) - identical.</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       <c r="N34" s="2"/>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - only one bar was clicked in this run.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: clicking a different bar replaced the heading with the new month and reset the table footer to '1-15 of 36', confirming the paging reset.</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Paymentus account available.</t>
+          <t xml:space="preserve">QA 2026-09-15 Paymentus: CONFIRMED. Two POSTs fired - the first with page_size 15, the second automatically with page_size 198 matching totalRecord, so the summary counts cover the whole month.</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Paymentus account available.</t>
+          <t xml:space="preserve">QA 2026-09-15 Paymentus: all three cards rendered - Ach (29), Token (246), Card (63) - each with a currency-formatted value.</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14 SnapPay Apr 2026: 3 + 52 = 55 and the table footer read '1-15 of 55'. Counts reconcile. Written against Paymentus but the reconciliation held on SnapPay.</t>
+          <t xml:space="preserve">QA 2026-09-15 Paymentus: card counts matched the tooltip exactly for the same month (29 / 246 / 63). Note the drill-down table holds 198 rows because it is filtered to Sale requests, so it is not expected to equal the sum of the cards.</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14 SnapPay: all four controls present (first / previous / next / last page). Paging itself not driven.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: the next-page control moved the footer from '1-15 of 55' to '16-30 of 55'. First/previous/last were present but only next was driven.</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       <c r="N46" s="2"/>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: switching rows per page from 15 to 25 re-rendered 25 rows, moved the footer to '1-25 of 55' and sent page_size 25.</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       <c r="N47" s="2"/>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - the duplicate-request question is still open.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: from page 2 ('26-50 of 55') switching back to 15 returned the table AND the pagination control to page 1 ('1-15 of 55'). Confirmed the duplicate-request behaviour - the single action fired TWO transaction POSTs, both with page_number 1.</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
       <c r="N49" s="2"/>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="S49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14 SnapPay: timestamps rendered as '4/30/2026, 11:30:39 AM' but no cross-check against the Transactions module was done.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: timestamps render in the viewer's locale format (e.g. '4/30/2026, 11:30:39 AM'). The conversion against a different profile timezone was not cross-checked, so treat the timezone half as unproven.</t>
         </is>
       </c>
     </row>
@@ -5014,7 +5014,7 @@
       <c r="N50" s="2"/>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="S50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - download not triggered in this run.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: 'Export to Excel' downloaded a file named Transactions.xls.</t>
         </is>
       </c>
     </row>
@@ -5113,7 +5113,7 @@
       <c r="N51" s="2"/>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="S51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: 'Export to Pdf' downloaded a file named paymentTrendsTable.pdf.</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       <c r="N52" s="2"/>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="S52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: with 25 rows on screen the exported file contained exactly 25 data rows - the export covers the current page only, not the whole month.</t>
         </is>
       </c>
     </row>
@@ -5408,7 +5408,7 @@
       <c r="N54" s="2"/>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -5428,7 +5428,7 @@
       </c>
       <c r="S54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: clicking refresh issued a fresh periodic_payment_stats_us request and the chart redrew.</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       <c r="N55" s="2"/>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -5526,7 +5526,7 @@
       </c>
       <c r="S55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: the refresh request carried the same pageSize as the selected range, so the range is preserved.</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       <c r="N56" s="2"/>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="S56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - still worth confirming with the product owner.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: CONFIRMED - the drill-down was still open after refresh. Only changing the time range clears it. Confirm with the product owner whether that is intended.</t>
         </is>
       </c>
     </row>
@@ -5822,7 +5822,7 @@
       </c>
       <c r="S58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: corrupting the stored token and forcing a refresh did NOT redirect to sign-in - the page stayed on /paymenttrends and the corrupted token remained in storage. It is not clear whether a request was actually made, so this is inconclusive rather than a confirmed failure. Re-test by letting a session expire naturally.</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="S64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: ANOMALY WORTH CHECKING MANUALLY. Clicking three different bars in quick succession left the drill-down showing the FIRST month clicked (Apr 2026), not the last. That is the stale-response risk this case is meant to catch, but the clicks were script-driven at speed and the later ones may have landed on shifted layout. Re-run this one by hand before raising it.</t>
         </is>
       </c>
     </row>
@@ -7282,7 +7282,7 @@
       <c r="N73" s="2"/>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corrected after run</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="S73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: CORRECTED - observed From Date 08/15/2026 12:00 AM against a To Date of 09/14/2026, i.e. today minus 30 days, NOT the 1st of the previous month. The module doc and my original case were both wrong.</t>
+          <t xml:space="preserve">QA 2026-09-15: re-confirmed on a second day - defaults read 08/16/2026 to 09/15/2026, exactly 30 days, not the 1st of the previous month.</t>
         </is>
       </c>
     </row>
@@ -7972,7 +7972,7 @@
       <c r="N80" s="2"/>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P80" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="S80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - date validation not driven in this run.</t>
+          <t xml:space="preserve">QA 2026-09-15 IPG: setting To Date earlier than From Date and pressing Submit produced the message 'Invalid date range' and fired zero stats requests.</t>
         </is>
       </c>
     </row>
@@ -8071,7 +8071,7 @@
       <c r="N81" s="2"/>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -8091,7 +8091,7 @@
       </c>
       <c r="S81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 IPG: setting From Date to a future date and pressing Submit fired zero stats requests and produced NO message of any kind - the silent rejection is confirmed, and it is inconsistent with the inverted-range case above.</t>
         </is>
       </c>
     </row>
@@ -8168,7 +8168,7 @@
       <c r="N82" s="2"/>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P82" s="2" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="S82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - calendar constraints are set in code but were not clicked through.</t>
+          <t xml:space="preserve">QA 2026-09-15 IPG: opening the From calendar and stepping to the current month showed 18 disabled days against 17 enabled - future dates are blocked. Navigation past the current month was also refused.</t>
         </is>
       </c>
     </row>
@@ -8265,7 +8265,7 @@
       <c r="N83" s="2"/>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P83" s="2" t="inlineStr">
@@ -8285,7 +8285,7 @@
       </c>
       <c r="S83" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 IPG: the To calendar opened on the current month; stepping back to the From month showed 21 disabled days against 21 enabled - dates before the selected From Date are blocked.</t>
         </is>
       </c>
     </row>
@@ -8660,7 +8660,7 @@
       <c r="N87" s="2"/>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P87" s="2" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="S87" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 IPG: clearing the From field left the placeholder showing and pressing Submit fired ZERO stats requests, so no blank range reaches the API.</t>
         </is>
       </c>
     </row>
@@ -8757,7 +8757,7 @@
       <c r="N88" s="2"/>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Corrected after run</t>
         </is>
       </c>
       <c r="P88" s="2" t="inlineStr">
@@ -8777,7 +8777,7 @@
       </c>
       <c r="S88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 IPG: CORRECTED - typing '13/45/2026 99:99 XX' is not rejected. The picker coerces it to a valid date (observed '03/04/2026 09:09 AM') and Submit then fires a normal request. The original expectation of 'no request is sent' was wrong; the page stays stable, which is the real point.</t>
         </is>
       </c>
     </row>
@@ -9252,7 +9252,7 @@
       <c r="N93" s="2"/>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P93" s="2" t="inlineStr">
@@ -9272,7 +9272,7 @@
       </c>
       <c r="S93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: the refresh icon's class changed on click, confirming the animation is applied. The exact spin class was not captured because it clears after about a second.</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9350,7 @@
       <c r="N94" s="2"/>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P94" s="2" t="inlineStr">
@@ -9370,7 +9370,7 @@
       </c>
       <c r="S94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: clicking the refresh icon collapsed the expanded Prepare Query panel.</t>
         </is>
       </c>
     </row>
@@ -9544,7 +9544,7 @@
       <c r="N96" s="2"/>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P96" s="2" t="inlineStr">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="S96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: three rapid Submit clicks produced three stats requests - there is no debouncing. The table stayed consistent with the selected range. Watch for a slow earlier response overwriting a newer one on a loaded environment.</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="S104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - header clicks not driven.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: clicking a column header changed nothing and no sort arrow appeared - but the grid was empty because of the page-wide 400, so this proves little. Re-test once PS-NEG-11 is fixed.</t>
         </is>
       </c>
     </row>
@@ -10626,7 +10626,7 @@
       <c r="N107" s="2"/>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P107" s="2" t="inlineStr">
@@ -10646,7 +10646,7 @@
       </c>
       <c r="S107" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised - panel not expanded in this run.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: panel was collapsed on load, expanded on click, and showed Select, Group, Having, And/Or, Execute and Cancel. 'Having 1' stays hidden until And/Or is chosen.</t>
         </is>
       </c>
     </row>
@@ -10723,7 +10723,7 @@
       <c r="N108" s="2"/>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P108" s="2" t="inlineStr">
@@ -10743,7 +10743,7 @@
       </c>
       <c r="S108" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: Select opened pre-populated with Funding Method, Funding Category, Channel and Displayed Fee Amount - and Group carries the same four by default.</t>
         </is>
       </c>
     </row>
@@ -10820,7 +10820,7 @@
       <c r="N109" s="2"/>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P109" s="2" t="inlineStr">
@@ -10840,7 +10840,7 @@
       </c>
       <c r="S109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: Select opened pre-populated with exactly Request Type, Channel, transaction Amount and Fee Amount.</t>
         </is>
       </c>
     </row>
@@ -10918,7 +10918,7 @@
       <c r="N110" s="2"/>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P110" s="2" t="inlineStr">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="S110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: removing every Select chip left 0 chips and the Execute button became disabled.</t>
         </is>
       </c>
     </row>
@@ -11016,7 +11016,7 @@
       <c r="N111" s="2"/>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P111" s="2" t="inlineStr">
@@ -11036,7 +11036,7 @@
       </c>
       <c r="S111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: clearing every Group chip left 0 chips, disabled the Having controls and disabled Execute.</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       <c r="N112" s="2"/>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P112" s="2" t="inlineStr">
@@ -11134,7 +11134,7 @@
       </c>
       <c r="S112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: Having field options were exactly Funding Method, Funding Category, Channel, Displayed Fee Amount; choosing the text field 'Funding Method' offered exactly two operators - 'is equal to' and 'is not equal to'.</t>
         </is>
       </c>
     </row>
@@ -11212,7 +11212,7 @@
       <c r="N113" s="2"/>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P113" s="2" t="inlineStr">
@@ -11232,7 +11232,7 @@
       </c>
       <c r="S113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: choosing the amount field 'Displayed Fee Amount' offered all six operators - is equal to, is not equal to, is greater than, is greater than and equal to, is less than, is less than and equal to.</t>
         </is>
       </c>
     </row>
@@ -11310,7 +11310,7 @@
       <c r="N114" s="2"/>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P114" s="2" t="inlineStr">
@@ -11330,7 +11330,7 @@
       </c>
       <c r="S114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: the And/Or control was disabled while the first Having row was incomplete.</t>
         </is>
       </c>
     </row>
@@ -11824,7 +11824,7 @@
       </c>
       <c r="S119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised, but the default query params were confirmed per gateway: IPG request_type; SnapPay request_type,channel,transaction_amount,fee_amount; CommerceHub payment_type; BillPay funding_method,funding_category,channel,displayed_fee_amount.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: pressing Execute with the DEFAULT chips sent select_fields and groupby_fields identically as 'request_type,channel,transaction_amount,fee_amount' - no mismatch on this path. The risk only arises if the amount field is removed and re-added from the Select dropdown, which re-reads a different option list. Re-test by removing and re-adding 'transaction Amount' before pressing Execute.</t>
         </is>
       </c>
     </row>
@@ -12481,7 +12481,7 @@
       <c r="N126" s="2"/>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P126" s="2" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="S126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Console output not captured in this run - worth doing while the 400 is still reproducible.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: CONFIRMED - the browser console shows 'err is not defined' alongside the 400. The failure handler throws its own ReferenceError, so the real API error never reaches the console. Also seen: repeated 'Invalid value used as weak map key' page errors.</t>
         </is>
       </c>
     </row>
@@ -13262,7 +13262,7 @@
       <c r="N134" s="2"/>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P134" s="2" t="inlineStr">
@@ -13282,7 +13282,7 @@
       </c>
       <c r="S134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: navigating to Payment Trends and back reset the From Date to the default 30-day window and left the Prepare Query panel collapsed - a clean state with no leftovers.</t>
         </is>
       </c>
     </row>
@@ -13584,7 +13584,7 @@
       </c>
       <c r="S137" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed. These create real payments on the shared QA environment, which needs your go-ahead first. The Payment Stats half is also blocked until PS-NEG-11 is fixed - with sub_merchant_id sent empty the page returns 400 and shows no figures to compare against.</t>
+          <t xml:space="preserve">QA 2026-09-15: the payment half of this flow is proven (see PA-E2E-03) and Virtual Terminal is a valid entry point - the payment is recorded as a 'Sale' request type and is picked up by the analytics filters. The Payment Stats half still cannot be checked while PS-NEG-11 leaves that page returning 400 with no figures.</t>
         </is>
       </c>
     </row>
@@ -13765,7 +13765,7 @@
       <c r="N139" s="2"/>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P139" s="2" t="inlineStr">
@@ -13785,7 +13785,7 @@
       </c>
       <c r="S139" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed. These create real payments on the shared QA environment, which needs your go-ahead first. The Payment Stats half is also blocked until PS-NEG-11 is fixed - with sub_merchant_id sent empty the page returns 400 and shows no figures to compare against.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: CONFIRMED end to end. Current-month tooltip read Token(12) Card(45) before the payment; a card payment was taken through Virtual Terminal &gt; Collect Payment; after refreshing, the same month read Token(12) Card(46) - the card count rose by exactly one and the token count did not move.</t>
         </is>
       </c>
     </row>
@@ -13865,7 +13865,7 @@
       <c r="N140" s="2"/>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P140" s="2" t="inlineStr">
@@ -13885,7 +13885,7 @@
       </c>
       <c r="S140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed. These create real payments on the shared QA environment, which needs your go-ahead first. The Payment Stats half is also blocked until PS-NEG-11 is fixed - with sub_merchant_id sent empty the page returns 400 and shows no figures to compare against.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: CONFIRMED. The new payment appeared on page 1 of the drill-down as request type 'CardSale' with the correct amount, the customer number used at payment time, a timestamp within a minute of the payment, and status SUCCESS. The footer total also rose by one.</t>
         </is>
       </c>
     </row>
@@ -14460,7 +14460,7 @@
       <c r="N146" s="2"/>
       <c r="O146" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P146" s="2" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="S146" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed. These create real payments on the shared QA environment, which needs your go-ahead first. The Payment Stats half is also blocked until PS-NEG-11 is fixed - with sub_merchant_id sent empty the page returns 400 and shows no figures to compare against.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: CONFIRMED. 'Export to Excel' produced Transactions.xls and the newly created payment was present in the exported rows.</t>
         </is>
       </c>
     </row>
@@ -14780,7 +14780,7 @@
       </c>
       <c r="S149" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not executed. These create real payments on the shared QA environment, which needs your go-ahead first. The Payment Stats half is also blocked until PS-NEG-11 is fixed - with sub_merchant_id sent empty the page returns 400 and shows no figures to compare against.</t>
+          <t xml:space="preserve">QA 2026-09-15: single-payment aggregation is proven by PA-E2E-03 (+1 exactly). The multi-payment sum still needs the Payment Stats amount column, which is blocked by PS-NEG-11.</t>
         </is>
       </c>
     </row>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">52</t>
+          <t xml:space="preserve">91</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -15288,7 +15288,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">91</t>
+          <t xml:space="preserve">52</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Correct PS-NEG-11: Payment Stats fails on refresh only, not   every request
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -7596,7 +7596,7 @@
       </c>
       <c r="S76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -7692,7 +7692,7 @@
       </c>
       <c r="S77" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -7795,7 +7795,7 @@
       </c>
       <c r="S78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -8388,7 +8388,7 @@
       </c>
       <c r="S84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -8485,7 +8485,7 @@
       </c>
       <c r="S85" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -8583,7 +8583,7 @@
       </c>
       <c r="S86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -8875,7 +8875,7 @@
       </c>
       <c r="S89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
       </c>
       <c r="S92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -9467,7 +9467,7 @@
       </c>
       <c r="S95" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -10065,7 +10065,7 @@
       </c>
       <c r="S101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -10162,7 +10162,7 @@
       </c>
       <c r="S102" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="S103" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="S104" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15 BillPay: clicking a column header changed nothing and no sort arrow appeared - but the grid was empty because of the page-wide 400, so this proves little. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: clicking a column header changed nothing and no sort arrow appeared - but the grid was empty because I had opened the page by URL, which drops the sub-merchant id (PS-NEG-11). Re-test by reaching Payment Stats from the sidebar so the table has rows to sort.</t>
         </is>
       </c>
     </row>
@@ -11429,7 +11429,7 @@
       </c>
       <c r="S115" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -11528,7 +11528,7 @@
       </c>
       <c r="S116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -11627,7 +11627,7 @@
       </c>
       <c r="S117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -11726,7 +11726,7 @@
       </c>
       <c r="S118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12015,7 +12015,7 @@
       </c>
       <c r="S121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12112,7 +12112,7 @@
       </c>
       <c r="S122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12208,7 +12208,7 @@
       </c>
       <c r="S123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12305,7 +12305,7 @@
       </c>
       <c r="S124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
       </c>
       <c r="S128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12795,7 +12795,7 @@
       </c>
       <c r="S129" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12893,7 +12893,7 @@
       </c>
       <c r="S130" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -12989,7 +12989,7 @@
       </c>
       <c r="S131" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -13087,7 +13087,7 @@
       </c>
       <c r="S132" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -13184,7 +13184,7 @@
       </c>
       <c r="S133" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: blocked by the page-wide 400 - payment_stats_us is rejected for every gateway because sub_merchant_id is sent empty, so no data ever renders. Re-test once PS-NEG-11 is fixed.</t>
+          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
         </is>
       </c>
     </row>
@@ -13307,35 +13307,37 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stats request must carry the active sub-merchant identifier</t>
+          <t xml:space="preserve">Payment Stats keeps its data after a page refresh</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Network tab open</t>
+          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Network tab open, filtered on payment_stats</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every payment_stats_us call must include a populated sub_merchant_id
-The backend rejects the call outright when it is missing
+          <t xml:space="preserve">Reach the page two ways and compare:
+  (a) click Payment Analytics &gt; Payment Stats in the sidebar
+  (b) press F5 on that same page, or paste the /paymentStats URL into a fresh tab
+Watch the sub_merchant_id query parameter on each request
 Gateway: any - behaviour is identical on every gateway</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Open DevTools &gt; Network and filter on payment_stats
-2. Navigate to Payment Stats
-3. Inspect the outgoing request query string
-4. Find the sub_merchant_id parameter
-5. Verify it carries the identifier of the sub-merchant selected in the portal header, and is not blank
-6. Verify the response is HTTP 200 and the table populates
-7. Repeat for IPG, BillPay, SnapPay, CommerceHub, MerchantE and NuveiPaya</t>
+          <t xml:space="preserve">1. Log in and open DevTools &gt; Network, filtering on 'payment_stats'
+2. Navigate to Payment Analytics &gt; Payment Stats using the sidebar
+3. Inspect the payment_stats_us request and verify sub_merchant_id carries the id shown in the portal header
+4. Verify the response is 200 and the table renders its payment-type rows
+5. Now press F5 to refresh that same page
+6. Inspect the new payment_stats_us request and verify sub_merchant_id is still populated
+7. Verify the response is still 200 and the table still shows its rows</t>
         </is>
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sub_merchant_id must be populated on every request and the call must return 200 with data. A blank value makes the backend reject the call and leaves the page permanently empty (defect, log it)</t>
+          <t xml:space="preserve">The page must load its data whichever way it is reached. A refresh that sends an empty sub_merchant_id, returns 400 and empties the table - with no error shown to the user - is a defect (log it)</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -13381,7 +13383,7 @@
       </c>
       <c r="S135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14: CONFIRMED and this is the headline defect. sub_merchant_id was sent EMPTY on every payment_stats_us request for IPG, BillPay, SnapPay and CommerceHub, and the backend rejects it with HTTP 400 ('sub_merchant_id is required'). Payment Stats therefore shows no data for any gateway on QA. Root cause: the mount effect fires the request before the sub-merchant is known and marks the range as already set, which permanently blocks the follow-up effect that would have re-fetched with a valid id.</t>
+          <t xml:space="preserve">QA 2026-09-14: CONFIRMED, and the trigger is a page refresh - NOT every request as first recorded. Navigating to Payment Stats from the sidebar sends a populated sub_merchant_id and the table renders normally. Pressing F5 on that same page re-sends it EMPTY, the backend returns 400 and the table empties with no error shown. Confirmed independently by the user in a normal browser session.</t>
         </is>
       </c>
     </row>
@@ -13584,7 +13586,7 @@
       </c>
       <c r="S137" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15: the payment half of this flow is proven (see PA-E2E-03) and Virtual Terminal is a valid entry point - the payment is recorded as a 'Sale' request type and is picked up by the analytics filters. The Payment Stats half still cannot be checked while PS-NEG-11 leaves that page returning 400 with no figures.</t>
+          <t xml:space="preserve">QA 2026-09-15: the payment half of this flow is proven (see PA-E2E-03) and Virtual Terminal is a valid entry point - the payment is recorded as a 'Sale' request type and is picked up by the analytics filters. The Payment Stats half is testable by navigating from the sidebar - just do not refresh the page, see PS-NEG-11.</t>
         </is>
       </c>
     </row>
@@ -14780,7 +14782,7 @@
       </c>
       <c r="S149" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15: single-payment aggregation is proven by PA-E2E-03 (+1 exactly). The multi-payment sum still needs the Payment Stats amount column, which is blocked by PS-NEG-11.</t>
+          <t xml:space="preserve">QA 2026-09-15: single-payment aggregation is proven by PA-E2E-03 (+1 exactly). The multi-payment sum needs the Payment Stats amount column, which renders fine when the page is reached from the sidebar.</t>
         </is>
       </c>
     </row>
@@ -15792,7 +15794,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Payment Stats is broken for every gateway</t>
+          <t xml:space="preserve">Payment Stats loses its data on refresh</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -15802,7 +15804,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sub_merchant_id sent empty on every request; backend returns 400</t>
+          <t xml:space="preserve">reached from the sidebar it works; a refresh or direct URL sends an empty sub_merchant_id and returns 400</t>
         </is>
       </c>
     </row>
@@ -15819,7 +15821,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">the 400 produces no toast, no banner, no message</t>
+          <t xml:space="preserve">the refresh 400 produces no toast, no banner, no message - it looks like a merchant with no payments</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Column cases: assert presence, not order
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -9710,12 +9710,13 @@
 6. Verify 'Qty'
 7. Verify 'Qty(%)'
 8. Repeat steps 1 to 7 as a CommerceHub merchant
-9. Repeat steps 1 to 7 as a NuveiPaya merchant</t>
+9. Repeat steps 1 to 7 as a NuveiPaya merchant
+10. Note: the columns need not appear in any particular order — only that all five are present</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">All three standard gateways show exactly Type, Amount, Amount(%), Qty and Qty(%) in that order</t>
+          <t xml:space="preserve">All three standard gateways show all five columns — Type, Amount, Amount(%), Qty and Qty(%). Column order is not asserted: reordering them changes nothing for the merchant</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -9819,7 +9820,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BillPay shows exactly those six columns in that order - a completely different set from IPG</t>
+          <t xml:space="preserve">BillPay shows all six columns — a completely different set from IPG. Order is not asserted: reordering them changes nothing for the merchant</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -9922,7 +9923,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SnapPay shows exactly those five columns in that order</t>
+          <t xml:space="preserve">SnapPay shows all five columns. Order is not asserted</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">

</xml_diff>

<commit_message>
PT-DRILL-11: count from UI, amounts from the periodic stats   response
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -10783,40 +10783,49 @@
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every month bar drills down and reconciles with the Transactions module</t>
+          <t xml:space="preserve">Every month bar drills down and reconciles for count and amount</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MerchantE customer-portal user authenticated; Payment Analytics group visible in sidebar; Payment Trends page reachable; Transactions module accessible for the same merchant</t>
+          <t xml:space="preserve">MerchantE customer-portal user authenticated; Payment Analytics group visible in sidebar; Payment Trends page reachable; Transactions module accessible for the same merchant; DevTools Network tab open</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Walk EVERY bar in the chart, not just one
-Compare per month: transaction count AND total amount
-Transactions filter: date between the 1st and last day of that month, plus the authorised/successful status for that gateway (BillPay: Authorization Status = Authorized)
+          <t xml:space="preserve">Walk EVERY bar in the chart, not just one.
+Where each figure comes from:
+  COUNT  - read from the UI. The screen is the only place it is shown: the hover tooltip,
+           the number in brackets on each summary card, and the table footer total.
+  AMOUNT - read from the periodic_payment_stats_us response. There is NO month total on
+           screen, so take the per-type amounts from the response for the selected month:
+             sumOfSuccessCardPayment  -&gt; the card amount
+             sumOfSuccessAchPayment   -&gt; the ACH amount
+Transactions filter: date between the 1st and last day of that month, plus the authorised/
+successful status for that gateway (BillPay: Authorization Status = Authorized)
 Gateway: any - behaviour is identical on every gateway</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Open Payment Trends with the default Last 6 Months range
-2. Take the left-most bar first, then work across to the right
-3. Hover the bar and note the counts shown in the tooltip
-4. Click it and verify 'Selected Month' names that same month
-5. Note the count in brackets on each summary card, and the amount beneath it
-6. Note the record total in the transaction table footer
-7. Open the Transactions module and filter to that month with the authorised status
-8. Verify the transaction count there matches the drill-down footer total
-9. Verify the total amount there matches the sum of the summary card amounts
-10. Repeat steps 3 to 9 for every remaining bar in the chart
-11. Verify a month whose bar has no height opens an empty drill-down rather than an error</t>
+          <t xml:space="preserve">1. Open DevTools &gt; Network and filter on 'periodic', then open Payment Trends
+2. Keep the periodic_payment_stats_us response open - it carries one entry per month
+3. Take the left-most bar first, then work across to the right
+4. Hover the bar and note the Card and ACH counts from the tooltip
+5. Click the bar and verify 'Selected Month' names that same month
+6. Note the count in brackets on each summary card, and the record total in the table footer
+7. In the response, find that month's entry and read sumOfSuccessCardPayment and sumOfSuccessAchPayment
+8. Open the Transactions module and filter to that month with the authorised status
+9. Verify the transaction count there matches the count shown on screen for that month
+10. Verify the card total there matches sumOfSuccessCardPayment for that month
+11. Verify the ACH total there matches sumOfSuccessAchPayment for that month
+12. Repeat steps 4 to 11 for every remaining bar in the chart
+13. Verify a month whose bar has no height opens an empty drill-down rather than an error</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every month in the range drills down to its own figures, and both the count and the amount match the Transactions module for that month. One month disagreeing while the others match points at that month's data rather than the page (log it with the month named)</t>
+          <t xml:space="preserve">For every month in the range: the count on screen matches the Transactions module, and the card and ACH amounts in the periodic stats response match the same totals there. One month disagreeing while the others match points at that month's data rather than the page (log it with the month named)</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -10847,7 +10856,7 @@
       </c>
       <c r="P109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">@PaymentAnalytics @PaymentTrends @allGateways @dataintegrity @regression</t>
+          <t xml:space="preserve">@PaymentAnalytics @PaymentTrends @allGateways @api @dataintegrity @regression</t>
         </is>
       </c>
       <c r="Q109" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Reword PS-NEG-02: only surfaces on a failed request
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -6135,38 +6135,44 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Browser console shows a secondary error when the stats request fails</t>
+          <t xml:space="preserve">Failure handler hides the real API error when a stats request fails</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Console open; ability to fail the stats request</t>
+          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Console open; ability to block or fail the stats request</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The failure handler itself throws, masking the original error
+          <t xml:space="preserve">This only shows up on a FAILED request. A healthy session never enters the failure handler,
+so the console stays clean apart from unrelated page noise ('Invalid value used as weak map key',
+which appears on every page regardless).
+To see it you must make the stats call fail - block payment_stats_us in DevTools, or use a
+merchant whose record is broken.
 Gateway: any - behaviour is identical on every gateway</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Open DevTools &gt; Console and clear it
-2. Block the payment_stats_us request
-3. Navigate to Payment Stats and let the request fail
-4. Read the console output
-5. Verify whether the real API error is logged
-6. Note any reference error raised by the handler itself instead of the underlying cause</t>
+2. Open Payment Stats normally first and confirm the console shows no reference error - this is
+   the control, and proves the next step is caused by the failure and not by the page itself
+3. Now block the payment_stats_us request in DevTools
+4. Reload Payment Stats and let the request fail
+5. Read the console output
+6. Verify the real API error reaches the console
+7. Note any reference error thrown by the handler itself in place of the underlying cause</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The genuine API error should reach the console. A handler that throws its own error and hides the real cause makes support diagnosis impossible (defect, log it)</t>
+          <t xml:space="preserve">When a stats request fails, the genuine API error must reach the console. A handler that throws its own reference error and swallows the real cause leaves support with nothing to diagnose (defect, log it). Note this is invisible during normal use - it only appears once something has already gone wrong</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t xml:space="preserve">Medium</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -16211,7 +16217,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">89</t>
+          <t xml:space="preserve">88</t>
         </is>
       </c>
       <c r="C53" s="2"/>
@@ -16224,7 +16230,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">42</t>
+          <t xml:space="preserve">43</t>
         </is>
       </c>
       <c r="C54" s="2"/>

</xml_diff>

<commit_message>
Renumber PS-SUB to close the gap left by the removed case
PS-SUB-02 to 08 become PS-SUB-01 to 07. The scenarios are unchanged; only the
identifiers move, so the section reads 01 to 07 with no gap where the removed
case used to sit.

  PS-SUB-01  Submit button stays enabled even when a date is missing
  PS-SUB-02  Refresh icon resets the date range back to the last-month window
  PS-SUB-03  Refresh icon spins while the request is in flight
  PS-SUB-04  Refresh closes the Prepare Query panel if it is open
  PS-SUB-05  Refresh restores the full column set after a custom query narrowed it
  PS-SUB-06  Repeated Submit clicks do not stack duplicate requests
  PS-SUB-07  Client request identifier sent with every stats call is fixed

The automation map and the verification evidence were remapped with them, so no
case carries another case's history.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -1841,7 +1841,7 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-17 IPG: Ctrl+A then Delete empties From Date, which falls back to showing 'MM/DD/YYYY hh:mm aa'. The table kept its data and Submit is NOT disabled (that is PS-SUB-02). OPEN QUESTION, PARKED 2026-09-17 - the expected result as written may be wrong. It says no request is sent with an empty date. In a page state where Submit is live, a request IS sent, and it carries the PREVIOUS date rather than an empty one: the field showed the placeholder while the request went out with fromDate=2026-08-01. The picker's onChange bails on a null value (index.js:546) so the stored date is never cleared - the merchant sees a blank box but gets figures for a range they cannot see. Whether no request is sent depends on whether Submit is live, which is the PS-SUB-01 gate. Case and test both left as they are for now.</t>
+          <t xml:space="preserve">QA 2026-09-17 IPG: Ctrl+A then Delete empties From Date, which falls back to showing 'MM/DD/YYYY hh:mm aa'. The table kept its data and Submit is NOT disabled (that is PS-SUB-01). OPEN QUESTION, PARKED 2026-09-17 - the expected result as written may be wrong. It says no request is sent with an empty date. In a page state where Submit is live, a request IS sent, and it carries the PREVIOUS date rather than an empty one: the field showed the placeholder while the request went out with fromDate=2026-08-01. The picker's onChange bails on a null value (index.js:546) so the stored date is never cleared - the merchant sees a blank box but gets figures for a range they cannot see. Whether no request is sent depends on whether Submit is live, which is the same Isdateset gate that makes the first click after page load do nothing. Case and test both left as they are for now.</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-02</t>
+          <t xml:space="preserve">PS-SUB-01</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-02
+          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-01
 Clears From Date and asserts Submit is disabled, then inverts the range and asserts the same. Marked test.fail(): the button is never disabled because index.js:606 has the disabled prop commented out.</t>
         </is>
       </c>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-03</t>
+          <t xml:space="preserve">PS-SUB-02</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-03
+          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-02
 Widens the window to six months and submits, then clicks refresh and asserts both dates return to the default 30-day window, the icon spins, and the table reloads with no more payments than the wider window held.</t>
         </is>
       </c>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-04</t>
+          <t xml:space="preserve">PS-SUB-03</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2305,7 +2305,7 @@
         <is>
           <t xml:space="preserve">1. Open Payment Stats from the sidebar and let the data load fully
 2. Click the refresh icon ONCE
-3. Verify it does NOT animate - the first click after page load is swallowed (see PS-SUB-01, same cause)
+3. Verify it does NOT animate - the first click after the page loads is swallowed
 4. Click the refresh icon a SECOND time
 5. Verify it now animates while the data reloads
 6. Verify the animation stops once the figures come back
@@ -2339,7 +2339,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-04
+          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-03
 Lets the page settle, clicks refresh and asserts the icon starts spinning. Marked test.fail(): on a freshly loaded page refresh does nothing at all.</t>
         </is>
       </c>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-17 IPG, DEFECT CONFIRMED, wording corrected after re-measurement. The refresh icon is not dead - it ignores exactly one click, the first after page load. Sampling the icon class every 40ms: click 1 never span and sent no request, click 2 span and returned HTTP 200, click 3 the same. An earlier note said it 'only works once a Submit has run' - that is wrong, a second refresh click is enough on its own. Same !Isdateset gate as PS-SUB-01, and one fix clears both.</t>
+          <t xml:space="preserve">QA 2026-09-17 IPG, DEFECT CONFIRMED, wording corrected after re-measurement. The refresh icon is not dead - it ignores exactly one click, the first after page load. Sampling the icon class every 40ms: click 1 never span and sent no request, click 2 span and returned HTTP 200, click 3 the same. An earlier note said it 'only works once a Submit has run' - that is wrong, a second refresh click is enough on its own. The cause is the !Isdateset gate: the handler clears the flag and then reads it on the next line, before React has applied the change.</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-05</t>
+          <t xml:space="preserve">PS-SUB-04</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-05
+          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-04
 Expands Prepare Query on BillPay, confirms Select, Group and Having plus Execute and Cancel, then asserts refresh collapses the panel and leaves the default columns intact.</t>
         </is>
       </c>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-06</t>
+          <t xml:space="preserve">PS-SUB-05</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-06
+          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-05
 Trims the Select list to two fields and executes, asserts the table narrows to those plus Amount and Count and that a dropped column really left, then asserts refresh restores the full default set.</t>
         </is>
       </c>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-07</t>
+          <t xml:space="preserve">PS-SUB-06</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-07
+          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-06
 Records the figures for a 3-day and a 90-day range separately, then fires the 90-day query and switches to the 3-day range without waiting, so two different queries are in flight at once. Asserts the newest one wins. Replaces an earlier version that clicked Submit three times on the SAME range - every request asked for the same figures, so it could never fail.</t>
         </is>
       </c>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-08</t>
+          <t xml:space="preserve">PS-SUB-07</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-08
+          <t xml:space="preserve">payment-analytics.spec.ts :: @PS-SUB-07
 Collects clientRequestId from two separate calls and asserts they differ. Marked test.fail(): the value is hard-coded. One of only three network reads in the module - the parameter has no UI surface.</t>
         </is>
       </c>
@@ -15641,7 +15641,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-LOAD-06 (flag=SUCCESS), PS-SUB-08 (clientRequestId) and PT-LOAD-07 (pageNumber). Each is a query parameter that is never displayed, never configurable and leaves no visible trace, so the screen genuinely cannot answer the question. Every other case is checked on screen</t>
+          <t xml:space="preserve">PS-LOAD-06 (flag=SUCCESS), PS-SUB-07 (clientRequestId) and PT-LOAD-07 (pageNumber). Each is a query parameter that is never displayed, never configurable and leaves no visible trace, so the screen genuinely cannot answer the question. Every other case is checked on screen</t>
         </is>
       </c>
     </row>
@@ -16518,7 +16518,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-02</t>
+          <t xml:space="preserve">PS-SUB-01</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -16535,7 +16535,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-04</t>
+          <t xml:space="preserve">PS-SUB-03</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -16552,7 +16552,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PS-SUB-08</t>
+          <t xml:space="preserve">PS-SUB-07</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Record results for the five cases still marked not verified
PS-DATE-03, PS-PQ-10, PS-PQ-11 and PS-PQ-12 pass; PS-PQ-13 behaves as
recorded and stays expected-fail. Their remarks still read 'Not exercised in
this run', which has not been true for some time.

PS-PQ-10 and PS-PQ-11 note that they are proven on screen rather than by
reading the request: a query that reaches the API wrongly shows up in the
table, which is what the merchant relies on.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -1512,7 +1512,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
+          <t xml:space="preserve">QA 2026-09-22 PASS. Changing the From Date and pressing Submit refetches: the pickers hold the new range and both the table and the graph redraw to match it.</t>
         </is>
       </c>
     </row>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
+          <t xml:space="preserve">QA 2026-09-22 PASS on BillPay. Trimming Select to two fields and pressing Execute rebuilds the table around exactly those fields plus Amount and Count; the dropped fields disappear as columns and the rows regroup, so fewer rows carry larger counts. Proven on screen - the DevTools step is not needed, since a query that reaches the API wrongly shows up in the table.</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
+          <t xml:space="preserve">QA 2026-09-22 PASS on BillPay. A Having clause of Funding Method is equal to a value present in the data returns only rows carrying that value, and fewer rows than the unfiltered table. Proven on screen rather than by reading having_fields: a clause that works shows itself in the rows, which is what the merchant relies on.</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
+          <t xml:space="preserve">QA 2026-09-22 PASS on BillPay. Cancel collapses the panel, restores the default columns and puts the default date range back.</t>
         </is>
       </c>
     </row>
@@ -4925,7 +4925,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Verified</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not exercised in this run. NOTE: this case IS testable today - reach Payment Stats by clicking through the sidebar, not by opening the URL directly. A direct load or refresh drops the sub-merchant id and returns 400 (see PS-NEG-11), which is what my probes hit.</t>
+          <t xml:space="preserve">QA 2026-09-22 DEFECT CONFIRMED, behaves as recorded. Cancel restores what is DISPLAYED but not the underlying query state, so an Execute straight after Cancel sends the query the panel no longer shows. Test asserts the intended behaviour and is marked expected-fail.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite PS-PQ-11 and PS-PQ-16 to match what they actually verify
PS-PQ-11 was written as a DevTools check — scenario, steps and expected result
all turned on reading having_fields. The clause is judged by the rows it
returns instead: one that reaches the backend wrongly shows up as wrong rows,
which is what the merchant relies on. Adds the two checks the old steps
lacked, that the result is smaller than unfiltered and not empty.

PS-PQ-16 was written around MerchantE returning an error and being blocked
until its merchant record was fixed. That premise no longer holds: the stats
request answers 200 and the panel is fully populated. What it does not do is
act on anything. The case now asks whether the panel drives the table, and
says to judge it by the columns, since the account has no payments and every
row reads $0.00.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -4658,7 +4658,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Having clause is sent to the API in the expected form</t>
+          <t xml:space="preserve">Having clause is applied to the rows, singly and when two are joined</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -4669,24 +4669,26 @@
       <c r="G45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Having: Funding Method is equal to a value present in the data
-Expected having_fields form: field then operator then the quoted value
+Second condition: another field, joined with And
+The clause is judged by the rows it returns, not by the request - a clause that reaches the backend wrongly shows up as wrong rows
 Gateway: BillPay</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Open Payment Stats as BillPay and expand Prepare Query
-2. Build a Having clause of 'Funding Method' 'is equal to' and a value you can see in the table
-3. Click Execute
-4. In DevTools inspect the having_fields query parameter
-5. Verify it carries the field name, the operator and the value in quotes
-6. Verify the returned rows all satisfy that condition
-7. Add a second condition joined by And and verify both appear in having_fields</t>
+2. Note the values shown in the Funding Method column and how many rows there are
+3. Build a Having clause of 'Funding Method' 'is equal to' a value you can see in the table
+4. Click Execute
+5. Verify every returned row carries that value and nothing else
+6. Verify the result is smaller than the unfiltered table, and not empty
+7. Choose And and add a second condition on a different field
+8. Click Execute and verify every row satisfies BOTH conditions</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Having clause reaches the API in the documented form and the returned rows all satisfy it, including when two conditions are joined</t>
+          <t xml:space="preserve">Each Having condition is applied to the rows returned, and two conditions joined by And return only the rows that satisfy both</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -5178,28 +5180,29 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MerchantE Prepare Query returns data once its merchant record is fixed</t>
+          <t xml:space="preserve">MerchantE Prepare Query panel drives the table</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MerchantE customer-portal user authenticated; Payment Analytics group visible in sidebar; Payment Stats page reachable; MerchantE credentials that resolve to a working merchant record</t>
+          <t xml:space="preserve">MerchantE customer-portal user authenticated; Payment Analytics group visible in sidebar; Payment Stats page reachable</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">MerchantE offers Prepare Query (it is in the SnapPay-like group)
 Select field options: Request Type, Channel, transaction Amount, Fee Amount
-Blocked until MerchantE stops returning an error on QA - see PT-NEG-01
+The earlier premise that MerchantE returns an error no longer holds - the stats request answers 200 and the panel is fully populated. What it does not do is act on anything.
+The account has no payments in the window, so every row reads $0.00 - judge this case by whether the COLUMNS change, not by the figures
 Gateway: MerchantE</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Log in as the MerchantE merchant and open Payment Stats
-2. Verify the stats request returns 200, not an error
-3. Verify the table renders payment-type rows with real figures
-4. Expand Prepare Query and verify the Select list offers Request Type, Channel, transaction Amount and Fee Amount
+          <t xml:space="preserve">1. Log in as the MerchantE merchant and open Payment Stats from the sidebar
+2. Verify the stats request returns 200 and the table renders its payment-type rows
+3. Expand Prepare Query and verify the Select list offers Request Type, Channel, transaction Amount and Fee Amount
+4. Note the column headings currently shown in the table
 5. Reduce Select to two fields and click Execute
 6. Verify the table rebuilds with only those fields plus Amount and Count
 7. Build a Having clause and Execute - verify only matching rows come back
@@ -5208,7 +5211,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MerchantE loads its stats and its Prepare Query behaves like the other query gateways. While the merchant record is broken this case cannot run - record it as blocked rather than failed</t>
+          <t xml:space="preserve">MerchantE's Prepare Query behaves like the other query gateways: trimming Select changes the columns, a Having clause narrows the rows, and Cancel puts the defaults back</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Rewrite PS-PQ-13 around what is visible, and drop its wrong premise
The case assumed the Group list is left empty after Cancel and that
groupby_fields goes out empty, and its steps required DevTools to see it.
Neither holds. After Cancel the panel shows EVERY field selected, and Execute
returns the narrowed column set from before Cancel — the stale state is the
previous query, not an empty one.

That contradiction is visible in the column headings, so the case is now
judged there: note the headings, trim a field, Execute, Cancel, reopen and
confirm every field is selected, press Execute without changing anything, and
compare the headings against the start.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -4868,35 +4868,36 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Executing immediately after Cancel does not send an empty grouping</t>
+          <t xml:space="preserve">Execute straight after Cancel queries what the panel shows</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BillPay customer-portal user authenticated; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Network tab open</t>
+          <t xml:space="preserve">BillPay customer-portal user authenticated; Payment Analytics group visible in sidebar; Payment Stats page reachable</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">After Cancel the Group list is left empty internally
-Action: press Execute straight after Cancel without re-picking fields
+          <t xml:space="preserve">Action: press Execute straight after Cancel without re-picking any field
+Cancel restores what is DISPLAYED but not the query behind it, so the panel and the result disagree
+Judged by the column headings - the panel shows every field selected while the table comes back missing the ones trimmed before Cancel
 Gateway: BillPay</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Open Payment Stats as BillPay and expand Prepare Query
-2. Run any Execute, then click Cancel
-3. Without choosing any field again, inspect the Group control
-4. Press Execute
-5. In DevTools inspect groupby_fields on the outgoing request
-6. Verify it is not sent empty, and that the table does not break
-7. Record what the API returns if an empty grouping is sent</t>
+          <t xml:space="preserve">1. Open Payment Stats as BillPay and note the column headings shown
+2. Expand Prepare Query, remove one field from Select and click Execute
+3. Verify the table narrows - that column is gone
+4. Click Cancel and verify the original column headings come back
+5. Expand Prepare Query again and verify Select shows EVERY field selected
+6. Without changing anything, press Execute
+7. Compare the column headings against step 1 - they must match, because that is what the panel is showing</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Execute straight after Cancel must not send an empty grouping or produce a broken table. Record the request and response if it does (defect, log it)</t>
+          <t xml:space="preserve">Execute after Cancel queries the fields the panel is displaying. If the table comes back missing the field trimmed before Cancel, the panel and the query disagree and the merchant is shown a result they did not ask for (defect, log it)</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add PS-NEG-11, and correct the claim that the failure is silent
A page refresh re-sends the stats request with an empty sub_merchant_id, the
server answers 400 and the table empties to "No rows". Two SnapPay
screenshots: the populated table reached through the sidebar, then the same
page after F5.

CORRECTION. The record said nothing is shown to the user. That is wrong. A red
toast appears carrying the server's message, "sub_merchant_id is required".
It is useless to a merchant and leaks an internal parameter name, but it is
not silence.

The silence measured under PS-NEG-01 was for a BLOCKED request, where no
response arrives and the page's handler never runs. When the server does
answer with an error, its message is shown. Both rows in the sheet now say so,
and the report describes what is actually on screen.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -5951,7 +5951,7 @@
       </c>
       <c r="S57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-21 DEFECT CONFIRMED by automation. With payment_stats_us blocked, the table renders its five headers with no rows, the refresh icon is not spinning, and there is no toast, banner or inline message of any kind. A broken request is indistinguishable from a date range that had no payments. Test asserts that something tells the user, marked expected-fail until it does.</t>
+          <t xml:space="preserve">QA 2026-09-21 DEFECT CONFIRMED by automation. With payment_stats_us BLOCKED, so that no response arrives at all, the table renders its five headers with no rows, the refresh icon is not spinning, and there is no toast, banner or inline message of any kind. A broken request is indistinguishable from a date range that had no payments. Scope note added 2026-09-23: this silence applies to a blocked or failed connection. When the server DOES answer with an error, the page shows its message - see PS-NEG-11, where a 400 produces a 'sub_merchant_id is required' toast. Test asserts that something tells the user, marked expected-fail until it does.</t>
         </is>
       </c>
     </row>
@@ -6937,7 +6937,7 @@
       </c>
       <c r="S67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-21 DEFECT CONFIRMED by automation. Reaching Payment Stats through the sidebar sends a populated sub_merchant_id and the table renders. Pressing F5 on that same page re-sends the request with an EMPTY sub_merchant_id, the API answers 400 and the table empties - with nothing shown to the user, because the page fails silently (PS-NEG-01).</t>
+          <t xml:space="preserve">QA 2026-09-21 DEFECT CONFIRMED by automation, remark corrected 2026-09-23. Reaching Payment Stats through the sidebar sends a populated sub_merchant_id and the table renders. Pressing F5 on that same page re-sends the request with an EMPTY sub_merchant_id, the server answers 400 and the table empties to 'No rows'. CORRECTION: an earlier note said nothing is shown to the user. That is wrong - a red toast appears carrying the server's message, 'sub_merchant_id is required'. It is unhelpful to a merchant and leaks an internal parameter name, but it is not silence. The silent case is PS-NEG-01, where the request is blocked outright and no response arrives at all, so the page's handler never runs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop the DevTools steps from PS-NEG-11
The page names the missing parameter itself - a refresh raises a
"sub_merchant_id is required" toast and empties the table to "No rows" - so
reading the request added nothing.

The steps now check what is on screen: the table still has rows, no error
toast appears, and the sub-merchant selector still shows the same
sub-merchant. That last one is the telling part, because it proves the page
knows which sub-merchant it is on and simply does not send it.

Leaves PS-NEG-12 as the only case in the section that genuinely needs the
request: measured under an October clock, the malformed date is accepted with
a 200, no toast, and eight rows rendered, so nothing on screen reveals it.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -6866,32 +6866,32 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Network tab open, filtered on payment_stats</t>
+          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reach the page two ways and compare:
+          <t xml:space="preserve">Reach the page two ways and compare what is on screen:
   (a) click Payment Analytics &gt; Payment Stats in the sidebar
-  (b) press F5 on that same page, or paste the /paymentStats URL into a fresh tab
-Watch the sub_merchant_id query parameter on each request
+  (b) press F5 on that same page
+The page names the missing parameter itself in a toast, so the request does not need to be read
 Gateway: any - behaviour is identical on every gateway</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Log in and open DevTools &gt; Network, filtering on 'payment_stats'
-2. Navigate to Payment Analytics &gt; Payment Stats using the sidebar
-3. Inspect the payment_stats_us request and verify sub_merchant_id carries the id shown in the portal header
-4. Verify the response is 200 and the table renders its payment-type rows
-5. Now press F5 to refresh that same page
-6. Inspect the new payment_stats_us request and verify sub_merchant_id is still populated
-7. Verify the response is still 200 and the table still shows its rows</t>
+          <t xml:space="preserve">1. Log in and navigate to Payment Analytics &gt; Payment Stats using the sidebar
+2. Verify the table renders its rows, and note the sub-merchant shown in the selector at the top of the page
+3. Press F5 to refresh that same page
+4. Verify the table still shows its rows
+5. Verify no error toast appears
+6. Verify the sub-merchant selector still shows the same sub-merchant
+7. Navigate to the page from the sidebar again and verify the data returns</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The page must load its data whichever way it is reached. A refresh that sends an empty sub_merchant_id, returns 400 and empties the table - with no error shown to the user - is a defect (log it)</t>
+          <t xml:space="preserve">The page loads its data whichever way it is reached. A refresh that empties the table to 'No rows' and raises a 'sub_merchant_id is required' toast is a defect (log it) - the selector still shows the sub-merchant, so the page knows it and simply does not send it</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Give PS-NEG-01 and PS-NEG-02 a failure step that can actually be followed
Both cases said to block the stats request in DevTools. That blocks the exact
URL, and the stats URL carries a toDate timestamp that changes on every call,
so the rule stops matching and the request sails through - which is what
happened when the case was attempted by hand.

Both now use DevTools > Network > throttling set to Offline. One dropdown,
nothing to configure, and it reproduces both defects: no message appears
anywhere, and the console carries net::ERR_INTERNET_DISCONNECTED followed by
the handler's own 'err is not defined'. Blocking never produced that reference
error, so PS-NEG-02 could not be reproduced by hand at all before.

PS-NEG-01's expected result is corrected too. It said the table is left empty.
Measured with Offline, the table keeps the PREVIOUS range's figures, so the
screen reads as a normal result for dates it never loaded - worse than an
empty table, and the reason the silence matters.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -5882,30 +5882,32 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; ability to block or fail the stats request via DevTools request blocking</t>
+          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools open</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Simulated failure: payment_stats_us blocked or returning 500
+          <t xml:space="preserve">Simulated failure: the stats request cannot reach the server
+Easiest way to cause it - DevTools &gt; Network &gt; change the throttling dropdown from 'No throttling' to 'Offline'. One dropdown, nothing to configure. Request blocking also works but blocks the exact URL, and the stats URL carries a toDate timestamp that changes every call, so the rule stops matching
 Expected UI today: no message of any kind
 Gateway: any - behaviour is identical on every gateway</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Open DevTools and add a request-block rule for payment_stats_us
-2. Navigate to Payment Stats
-3. Watch the page while the request fails
+          <t xml:space="preserve">1. Open Payment Stats from the sidebar and let the figures load
+2. Open DevTools &gt; Network and set the throttling dropdown to 'Offline'
+3. Change a date and press Submit, so the page tries to fetch
 4. Verify the refresh icon stops spinning
-5. Verify NO error toast, banner or inline message appears
-6. Verify the table is left empty or showing stale data with no explanation
-7. Record that a failed load is indistinguishable from a range with no payments</t>
+5. Verify NO error toast, banner or inline message appears anywhere
+6. Verify what the table is left showing - it keeps the PREVIOUS figures, so the screen looks like a normal result for the new dates
+7. Set throttling back to 'No throttling' when finished
+8. Record that a failed load is indistinguishable from a successful one</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The page fails silently - a broken request looks exactly like an empty date range, leaving the user with no idea anything went wrong (defect, log it)</t>
+          <t xml:space="preserve">The page fails silently. Nothing tells the merchant the request failed, and the table keeps the figures from the previous range, so the screen reads as a normal result for dates it never loaded (defect, log it)</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -5981,34 +5983,31 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Console open; ability to block or fail the stats request</t>
+          <t xml:space="preserve">Customer-portal user authenticated on any gateway; Payment Analytics group visible in sidebar; Payment Stats page reachable; DevTools Console open</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">This only shows up on a FAILED request. A healthy session never enters the failure handler,
-so the console stays clean apart from unrelated page noise ('Invalid value used as weak map key',
-which appears on every page regardless).
-To see it you must make the stats call fail - block payment_stats_us in DevTools, or use a
-merchant whose record is broken.
+          <t xml:space="preserve">This only shows up on a FAILED request. A healthy session never enters the failure handler, so the console stays clean apart from unrelated page noise ('Invalid value used as weak map key', which appears on every page regardless).
+Easiest way to cause it - DevTools &gt; Network &gt; set throttling to 'Offline', then force a request. Confirmed to reproduce it: the console carries net::ERR_INTERNET_DISCONNECTED followed by the handler's own 'err is not defined'.
 Gateway: any - behaviour is identical on every gateway</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Open DevTools &gt; Console and clear it
-2. Open Payment Stats normally first and confirm the console shows no reference error - this is
-   the control, and proves the next step is caused by the failure and not by the page itself
-3. Now block the payment_stats_us request in DevTools
-4. Reload Payment Stats and let the request fail
+          <t xml:space="preserve">1. Open Payment Stats from the sidebar and let the figures load
+2. Open DevTools &gt; Console and clear it. Confirm no reference error is present - this is the control, and proves the next step is caused by the failure and not by the page
+3. In DevTools &gt; Network set the throttling dropdown to 'Offline'
+4. Change a date and press Submit, so the page tries to fetch
 5. Read the console output
-6. Verify the real API error reaches the console
-7. Note any reference error thrown by the handler itself in place of the underlying cause</t>
+6. Verify the genuine network or API error is reported
+7. Note any reference error thrown by the handler itself in place of the real cause
+8. Set throttling back to 'No throttling' when finished</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">When a stats request fails, the genuine API error must reach the console. A handler that throws its own reference error and swallows the real cause leaves support with nothing to diagnose (defect, log it). Note this is invisible during normal use - it only appears once something has already gone wrong</t>
+          <t xml:space="preserve">When a stats request fails, the genuine error must reach the console. A handler that throws its own reference error - 'err is not defined' - alongside it leaves support with the fault of the handler rather than the cause (defect, log it). Note this is invisible during normal use; it only appears once something has already gone wrong</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Payment Stats sheet: record the silent stale-table behaviour on PS-NEG-02, and log the merchantId=undefined 400 as an open observation
PS-NEG-02 now states the user-visible harm, which the remark was missing.
After a failed Submit the table keeps showing the previous results and no
message appears on screen, so the figures look like an answer to the new date
range. Confirmed against before/after browser screenshots. Also notes that the
first two console faults are logged at info/log level, so anyone filtering the
console on Errors only will not see them.

PS-OBS-01 is new and is deliberately not called a defect. A 400 on
/v1/merchant/ui_config with merchantId=undefined was seen in a real browser on a
healthy page, but it does not reproduce under token injection, where the
parameter always carried a real value. The row records what is proven, what is
only a hypothesis, and the steps needed to settle it.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -6053,7 +6053,7 @@
       </c>
       <c r="S58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-24 DEFECT CONFIRMED, detail expanded from a merchant's own console. With the connection cut the handler breaks three times over: 'err: TypeError: Cannot convert undefined or null to object' (Object.keys on undefined), 'err: TypeError: Cannot read properties of undefined (reading error_code)', and 'Uncaught (in promise) ReferenceError: err is not defined'. It reaches into a response object that does not exist, because the request never completed. CORRECTION to an earlier note: the real cause is NOT lost - the browser logs net::ERR_INTERNET_DISCONNECTED itself, two lines above. The problem is that the handler adds three red lines of its own, so whoever is diagnosing has five errors to sift and none of them come from the handler doing its job. Each of the three is asserted separately so a partial fix shows as progress.</t>
+          <t xml:space="preserve">QA 2026-09-24 DEFECT CONFIRMED. Verified twice and they agree: automated (connection cut in Playwright) and manually in the browser with DevTools &gt; Network &gt; Offline, with before/after screenshots. USER-VISIBLE HARM (the main point): after Submit fails, the table keeps showing the PREVIOUS results unchanged and no message appears anywhere on screen. Confirmed by comparing the two screenshots - From Date changed from 08/25/2026 to 07/24/2026, Submit pressed, request failed, and the same rows (ACH/CheckSale, DISCOVER/CreditSale, MASTERCARD/CreditSale...) are still listed. The merchant is left believing those figures answer the new date range. The only way to find out is to open DevTools. CONSOLE: the failure handler then breaks three times over: 'err: TypeError: Cannot convert undefined or null to object' (Object.keys on undefined), 'err: TypeError: Cannot read properties of undefined (reading error_code)', and 'Uncaught (in promise) ReferenceError: err is not defined'. It reaches into a response object that does not exist, because the request never completed. NOTE FOR ANYONE REPRODUCING: the first two are logged at info/log level, not error, so they carry no red icon and are invisible if the console filter is set to Errors only. The real cause is NOT lost - the browser logs net::ERR_INTERNET_DISCONNECTED itself, two lines above. Each of the three is asserted separately so a partial fix shows as progress.</t>
         </is>
       </c>
     </row>
@@ -15381,6 +15381,82 @@
       <c r="S152" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Not executed. These create real payments on the shared QA environment, which needs your go-ahead first. The Payment Stats half is also blocked until PS-NEG-11 is fixed - with sub_merchant_id sent empty the page returns 400 and shows no figures to compare against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2">
+        <v>152</v>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PS-OBS-01</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payment Stats</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S9. Incidental Observations</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A config call fails with 400 on page load because merchantId is sent as undefined</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer-portal user signed in through the UI (not token injection); DevTools open on the Network and Console tabs from before the first request</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No fault injected. A completely healthy session.
+Gateway seen on: IPG</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Open DevTools and select the Console tab, with the level filter left on Default levels
+2. Sign in to the customer portal through the sign-in form
+3. Open Payment Stats from Payment Analytics
+4. Read the console without applying any filter
+5. Switch to the Network tab and look for calls to /v1/merchant/ui_config
+6. Check the merchantId value in the query string of the first such call</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every request on a healthy page load carries a real merchant id and returns 2xx. No 400 appears in the console when nothing has gone wrong.</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Automated</t>
+        </is>
+      </c>
+      <c r="O153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observed, not confirmed</t>
+        </is>
+      </c>
+      <c r="Q153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IPG (seen); other gateways unchecked</t>
+        </is>
+      </c>
+      <c r="S153" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QA 2026-09-24 OBSERVED, NOT YET CONFIRMED AS A DEFECT - deliberately not called a bug yet. Spotted in a merchant&amp;#8217;s own DevTools console while reproducing PS-NEG-02, on a healthy page with nothing injected: "Failed to load resource: the server responded with a status of 400" against qaapi1.tillipay.com, with merchantId=undefined in the query string. WHAT IS PROVEN: the endpoint is GET /v1/merchant/ui_config?merchantId=&lt;id&gt;, and on a normal load it is called five times over, which is worth a look on its own. WHAT IS NOT PROVEN: the cause. It does NOT reproduce in automation - on repeated IPG runs the parameter always carried a real value (526971115880) and not one request failed. The difference is that the automation writes mainMerchantId into localStorage before the app starts, so the value is ready earlier than it would be after a real sign-in. That points at a start-up ordering problem, where the first ui_config call goes out before the merchant id has been set - but that is a hypothesis, not a measurement, and it should not be written up as a defect until someone has watched it happen. TO CONFIRM: sign in through the form rather than by injecting a token, watch the Network tab from the very first request, and see whether the first ui_config call carries undefined. IMPACT IF REAL: one failed config call on every fresh sign-in, and whatever ui_config drives is left to fall back on defaults. Not blocking - the page still loads and the figures are correct.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bring the PS-SUB-01 and PS-SUB-07 remarks up to what was actually measured
PS-SUB-01 said only that Submit is never disabled. Re-checking showed the button
also accepts the click: with From Date cleared the query runs and returns Card
Payments of $44,903.20 across 708 payments while the date box stays empty, with
nothing on the page saying what period that covers. Read as it stood, the row
sounded like a cosmetic styling problem.

PS-SUB-07 had IPG only. Adding BillPay a week later, with the same value, and
two requests in one session that differed in every other respect, shows the
value is fixed in the source rather than per-session or per-merchant. Also
records what the number is: 1647602068707 as a millisecond timestamp is
18 March 2022 11:14:28 UTC, a Date.now() result pasted in as a constant.

Both rows now point at their write-ups in PaymentStats_Bugs.docx. Priority,
automation status, verified state and expected results are unchanged.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -2158,7 +2158,7 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-17 IPG, DEFECT CONFIRMED with source evidence, expected result rewritten. Submit reported enabled in every state a merchant can actually reach: on load, and with From Date cleared entirely - the disabled attribute was absent throughout. (An inverted range was also tried, but only by typing a date past the picker's minimum; the To Date calendar greys out every day before the current From Date, so that state cannot be produced from the UI and is not part of this case.) The cause is not missing logic: isSubmitButtonDisabled is declared at index.js:86 and updated in five places, but the line that applies it is commented out at index.js:606 - // disabled={isSubmitButtonDisabled}. Uncommenting it is the whole fix.</t>
+          <t xml:space="preserve">QA 2026-09-17 IPG, DEFECT CONFIRMED with source evidence, expected result rewritten. Submit reported enabled in every state a merchant can actually reach: on load, and with From Date cleared entirely - the disabled attribute was absent throughout. (An inverted range was also tried, but only by typing a date past the picker's minimum; the To Date calendar greys out every day before the current From Date, so that state cannot be produced from the UI and is not part of this case.) The cause is not missing logic: isSubmitButtonDisabled is declared at index.js:86 and updated in five places, but the line that applies it is commented out at index.js:606 - // disabled={isSubmitButtonDisabled}. Uncommenting it is the whole fix. RE-CONFIRMED 2026-09-24 on IPG, and the finding goes further than first recorded. Submit is not only enabled - it accepts the click and the query runs. With From Date cleared entirely, pressing Submit returned a full result: Card Payments $44,903.20 across 708 payments, while the From Date box stayed empty. No message appeared and nothing on the page states what period those figures cover. That second half is the reason this matters: an enabled button that does nothing is an annoyance, but one that returns figures for an unstated period is something a merchant reads as an answer. Written up as defect 10 in PaymentStats_Bugs.docx with three marked screenshots.</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-17 IPG, DEFECT CONFIRMED. Every payment_stats_us call carried clientRequestId=1647602068707, the same fixed value on page load and after a date change, exactly as apis/payment.js:101 hard-codes it. Two requests cannot be told apart in logs or traced individually. This is one of only three places in the module where the test reads the network, because the parameter has no UI surface of any kind.</t>
+          <t xml:space="preserve">QA 2026-09-17 IPG, DEFECT CONFIRMED. Every payment_stats_us call carried clientRequestId=1647602068707, the same fixed value on page load and after a date change, exactly as apis/payment.js:101 hard-codes it. Two requests cannot be told apart in logs or traced individually. This is one of only three places in the module where the test reads the network, because the parameter has no UI surface of any kind. RE-CONFIRMED 2026-09-24 on BillPay - the same value 1647602068707, on a different merchant a week later, and on two requests within one session (a 30-day range and a 90-day range) that differed in every other respect. So the value is fixed in the source, not per-session or per-merchant. WHAT THE VALUE TELLS YOU: read as a millisecond timestamp, 1647602068707 is 18 March 2022 11:14:28 UTC - a Date.now() result from one development session pasted in as a constant instead of left as a call. The intent was right; only the call was replaced by its result. Worth checking whether the same literal was pasted elsewhere at the same time, and whether anything downstream has come to rely on it being fixed after four and a half years. Written up as defect 11 in PaymentStats_Bugs.docx, with no screenshots because the parameter has no UI surface.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Raise PS-NEG-02 to High and record why
The sheet said Medium while the write-up said High, so the two disagreed. High
is the right one. The harm is the same shape as PS-LOAD-10, already High: the
merchant is shown wrong figures with nothing saying so.

Three things decided it. There is no signal at all, so the merchant cannot
self-correct. The wrongness is total rather than a small gap, since every figure
on screen answers a different question from the one asked. And the trigger is
ordinary - a dropped connection or a VPN reconnect, not an exotic state.

Not raised to Critical because it needs a network failure first, whereas
PS-NEG-11 needs only a refresh and PS-NEG-12 needs only the calendar to reach
October. The reasoning is in the remark so the judgement can be argued with
rather than guessed at later.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -6012,7 +6012,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medium</t>
+          <t xml:space="preserve">High</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="S58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-24 DEFECT CONFIRMED. Verified twice and they agree: automated (connection cut in Playwright) and manually in the browser with DevTools &gt; Network &gt; Offline, with before/after screenshots. USER-VISIBLE HARM (the main point): after Submit fails, the table keeps showing the PREVIOUS results unchanged and no message appears anywhere on screen. Confirmed by comparing the two screenshots - From Date changed from 08/25/2026 to 07/24/2026, Submit pressed, request failed, and the same rows (ACH/CheckSale, DISCOVER/CreditSale, MASTERCARD/CreditSale...) are still listed. The merchant is left believing those figures answer the new date range. The only way to find out is to open DevTools. CONSOLE: the failure handler then breaks three times over: 'err: TypeError: Cannot convert undefined or null to object' (Object.keys on undefined), 'err: TypeError: Cannot read properties of undefined (reading error_code)', and 'Uncaught (in promise) ReferenceError: err is not defined'. It reaches into a response object that does not exist, because the request never completed. NOTE FOR ANYONE REPRODUCING: the first two are logged at info/log level, not error, so they carry no red icon and are invisible if the console filter is set to Errors only. The real cause is NOT lost - the browser logs net::ERR_INTERNET_DISCONNECTED itself, two lines above. Each of the three is asserted separately so a partial fix shows as progress.</t>
+          <t xml:space="preserve">QA 2026-09-24 DEFECT CONFIRMED. Verified twice and they agree: automated (connection cut in Playwright) and manually in the browser with DevTools &gt; Network &gt; Offline, with before/after screenshots. USER-VISIBLE HARM (the main point): after Submit fails, the table keeps showing the PREVIOUS results unchanged and no message appears anywhere on screen. Confirmed by comparing the two screenshots - From Date changed from 08/25/2026 to 07/24/2026, Submit pressed, request failed, and the same rows (ACH/CheckSale, DISCOVER/CreditSale, MASTERCARD/CreditSale...) are still listed. The merchant is left believing those figures answer the new date range. The only way to find out is to open DevTools. CONSOLE: the failure handler then breaks three times over: 'err: TypeError: Cannot convert undefined or null to object' (Object.keys on undefined), 'err: TypeError: Cannot read properties of undefined (reading error_code)', and 'Uncaught (in promise) ReferenceError: err is not defined'. It reaches into a response object that does not exist, because the request never completed. NOTE FOR ANYONE REPRODUCING: the first two are logged at info/log level, not error, so they carry no red icon and are invisible if the console filter is set to Errors only. The real cause is NOT lost - the browser logs net::ERR_INTERNET_DISCONNECTED itself, two lines above. Each of the three is asserted separately so a partial fix shows as progress. PRIORITY RAISED Medium -&gt; High on 2026-09-24, to match the write-up. The harm is the same shape as PS-LOAD-10, which is already High: the merchant is shown wrong figures with nothing saying so. Three things decided it - there is no signal at all, so the merchant cannot self-correct; the wrongness is total rather than a small gap, since every figure answers a different question from the one asked; and the trigger is ordinary, a dropped connection or a VPN reconnect. Not raised to Critical because it needs a network failure first, whereas PS-NEG-11 needs only a refresh and PS-NEG-12 needs only the calendar to reach October.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automate the two Paymentus cases, and mark the four India cases blocked
PT-LEG-03 and PT-TIP-03 are automated. Paymentus was recorded as blocked for
want of an account, but the entry was in credentials as active all along and
simply missing from the generated token pool. Regenerating the pool brought it
in, so both became runnable without anything being set up.

PT-LEG-04, PT-DRILL-07, PT-CARD-04 and PT-TBL-02 move from Not Automated to
Blocked. All four need an India merchant, and both India entries in the
credentials are active:false, so no token exists and nothing can run against
one. Confirmed that India is not being tested, so leaving them as Not Automated
was counting four cases as pending work that nobody is waiting on.

Payment Trends now stands at 23 of 70 automated, with PT-LOAD and PT-RANGE
complete, PT-LEG at three of four and PT-TIP at two of four.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -9143,7 +9143,7 @@
       </c>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Automated</t>
         </is>
       </c>
       <c r="N89" s="2"/>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="S89" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15 Paymentus: legend read ['Ach','Token','Card'] - the only gateway showing all three series. RENUMBERED 2026-09-25 from PT-LEG-07, so the block runs without gaps.</t>
+          <t xml:space="preserve">QA 2026-09-15 Paymentus: legend read ['Ach','Token','Card'] - the only gateway showing all three series. RENUMBERED 2026-09-25 from PT-LEG-07, so the block runs without gaps. AUTOMATED 2026-09-25 on the Paymentus account, which was in credentials as active but missing from the token pool until it was regenerated. Asserts the legend is exactly ['Ach','Token','Card'] - Paymentus is the only gateway drawing all three, so this is what stops PT-LEG-01 and PT-LEG-02's exact two-entry arrays being read as 'a legend may only ever have two series'. The legend is read with nothing hovered, because its selector also matches tooltip lines.</t>
         </is>
       </c>
     </row>
@@ -9243,13 +9243,13 @@
       </c>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Blocked</t>
         </is>
       </c>
       <c r="N90" s="2"/>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Blocked - no India account</t>
         </is>
       </c>
       <c r="P90" s="2" t="inlineStr">
@@ -9269,7 +9269,7 @@
       </c>
       <c r="S90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">India account not included in this token refresh. RENUMBERED 2026-09-25 from PT-LEG-08, so the block runs without gaps.</t>
+          <t xml:space="preserve">India account not included in this token refresh. RENUMBERED 2026-09-25 from PT-LEG-08, so the block runs without gaps. BLOCKED 2026-09-25 - no India merchant account. The india and indiaAdmin entries in credentials/qa.json are both active:false, so no token is generated and nothing can run against an India merchant. Confirmed with the user on 2026-09-25 that India is not being tested, so this is not pending work. Re-open only if an India account is activated.</t>
         </is>
       </c>
     </row>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Automated</t>
         </is>
       </c>
       <c r="N93" s="2"/>
@@ -9558,7 +9558,7 @@
       </c>
       <c r="S93" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15 Paymentus: tooltip showed Ach(29), Token(246) and Card(63) together.</t>
+          <t xml:space="preserve">QA 2026-09-15 Paymentus: tooltip showed Ach(29), Token(246) and Card(63) together. AUTOMATED 2026-09-25 on Paymentus. Asserts the tooltip carries exactly Ach, Token and Card, and that each count reads as a whole number rather than merely matching a text pattern. Measured on the day: Ach 29, Token 246, Card 63.</t>
         </is>
       </c>
     </row>
@@ -10317,13 +10317,13 @@
       </c>
       <c r="M101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Blocked</t>
         </is>
       </c>
       <c r="N101" s="2"/>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Blocked - no India account</t>
         </is>
       </c>
       <c r="P101" s="2" t="inlineStr">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="S101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">India account not included in this token refresh.</t>
+          <t xml:space="preserve">India account not included in this token refresh. BLOCKED 2026-09-25 - no India merchant account, same as PT-LEG-04. The india and indiaAdmin entries in credentials/qa.json are both active:false, so no token is generated and nothing can run against an India merchant. Confirmed with the user that India is not being tested, so this is not pending work. Re-open only if an India account is activated.</t>
         </is>
       </c>
     </row>
@@ -11112,13 +11112,13 @@
       </c>
       <c r="M109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Blocked</t>
         </is>
       </c>
       <c r="N109" s="2"/>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Blocked - no India account</t>
         </is>
       </c>
       <c r="P109" s="2" t="inlineStr">
@@ -11138,7 +11138,7 @@
       </c>
       <c r="S109" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">India account not included in this token refresh. RENUMBERED 2026-09-25 from PT-CARD-05, so the block runs without gaps.</t>
+          <t xml:space="preserve">India account not included in this token refresh. RENUMBERED 2026-09-25 from PT-CARD-05, so the block runs without gaps. BLOCKED 2026-09-25 - no India merchant account, same as PT-LEG-04. The india and indiaAdmin entries in credentials/qa.json are both active:false, so no token is generated and nothing can run against an India merchant. Confirmed with the user that India is not being tested, so this is not pending work. Re-open only if an India account is activated.</t>
         </is>
       </c>
     </row>
@@ -11405,13 +11405,13 @@
       </c>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Blocked</t>
         </is>
       </c>
       <c r="N112" s="2"/>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Blocked - no India account</t>
         </is>
       </c>
       <c r="P112" s="2" t="inlineStr">
@@ -11431,7 +11431,7 @@
       </c>
       <c r="S112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">India account not included in this token refresh.</t>
+          <t xml:space="preserve">India account not included in this token refresh. BLOCKED 2026-09-25 - no India merchant account, same as PT-LEG-04. The india and indiaAdmin entries in credentials/qa.json are both active:false, so no token is generated and nothing can run against an India merchant. Confirmed with the user that India is not being tested, so this is not pending work. Re-open only if an India account is activated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automate PT-TIP-04, measured rather than reasoned about
The case asks that the tooltip counts match the summary card counts for the same
month. An earlier reading of the code claimed the two come from different
sources and could legitimately differ, which would have made the case unsound
and a test of it a false-defect generator.

Measuring settled it. Hovering and clicking the same bar: wglUsa Ach 43 and Card
80, snapPay Token 19 and Card 92, paymentus Ach 29, Token 246 and Card 63 -
tooltip and cards identical on all three. The earlier reading was wrong.

IPG is deliberately excluded. There the tooltip read Ach 0 and Card 712 while
the cards read Ach 0 and Card 0. That is a genuine defect, but it is already
logged twice as PT-NEG-12 and PT-NEG-13, so running this case on IPG would fail
correctly while only re-reporting those.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -9628,7 +9628,7 @@
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Automated</t>
         </is>
       </c>
       <c r="N94" s="2"/>
@@ -9654,7 +9654,7 @@
       </c>
       <c r="S94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15 SnapPay: tooltip read Token(3) and Card(52); the summary cards for the same month read Token (3) and Card (52) - identical.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: tooltip read Token(3) and Card(52); the summary cards for the same month read Token (3) and Card (52) - identical. AUTOMATED 2026-09-25 on wglUsa, snapPay and paymentus. Measured first rather than reasoned about, by hovering and clicking the SAME bar: wglUsa Ach 43 / Card 80, snapPay Token 19 / Card 92, paymentus Ach 29 / Token 246 / Card 63 - tooltip and cards identical on all three. IPG IS DELIBERATELY EXCLUDED. There the tooltip read Ach 0 / Card 712 while the cards read Ach 0 / Card 0. That mismatch is a real defect but it is already logged twice, as PT-NEG-12 and PT-NEG-13, so running this case on IPG would fail correctly while only re-reporting those. CORRECTION to an earlier analysis: it was claimed the two numbers come from different sources and could legitimately differ, which would have made this case unsound. They agree on three of four gateways, so the case is sound and the earlier reading was wrong. Note for anyone extending it: hoverNewestMonthColumn() takes the newest bar and clickTallestBar() the tallest, so using them together compares two different months. hoverTallestBar() and pressAtPointer() were added to work on one bar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automate the Payment Stats half of PS-NEG-04, leaving the Transactions half manual
The case reconciles Payment Stats against Transactions for the same window. Only
the Stats side is automated; the test says so plainly and attaches the figures,
the window, the per-method breakdown and the manual steps to the run, so whoever
finishes it does not have to re-derive any of it.

The Transactions date filter works - proved by hand, 2019 returned 0 of 0 and
the last three months returned 542 against a 4,511 baseline. What could not be
done is driving it from a test. It is a MUI X v6 DatePicker with a segmented
field, and six approaches all left the date visible in the box while the request
carried no filter at all. The product is fine; the automation is not.

Runs on wglUsa rather than ipg. IPG draws the Card and ACH summary directly and
would have been simpler to read, but its Transactions side returns nothing
(PT-NEG-12), so the manual half would have had nothing to compare against.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -6225,13 +6225,13 @@
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Automated</t>
+          <t xml:space="preserve">Automated (partial)</t>
         </is>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not verified</t>
+          <t xml:space="preserve">Stats side verified; Transactions side manual</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="S60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-24 NO LONGER BLOCKED - the Transactions Date and Time filter works. The 2026-09-21 note below it is out of date. Verified by hand on WGL over both pages: on Payments, between 2019-01-01 and 2019-12-31 returned 0 of 0 while between 2026-06-23 and 2026-09-24 returned 542; on All Transactions the same two ranges returned 0 and 903 against a 4,511 baseline. The 'between' condition did not exist on 2026-09-21 and does now, so a fix appears to have landed alongside it. RECONCILE ON THE PAYMENTS PAGE, not All Transactions: Payment Stats counts payments, while All Transactions also carries refunds and voids. Both filter correctly, so this is a choice about what is being compared rather than about which one works. STILL PIN THE SUB-MERCHANT. Payment Stats defaults to 44052731 and reports card payments under it while All Transactions lists nothing at all for that sub-merchant, so both pages must be set to 44052730 before any comparison. That half of the original note still stands. NOT YET AUTOMATED, and the reason is worth knowing before anyone tries. The Payment Stats half is straightforward. The Transactions half could not be driven from Playwright on 2026-09-24: six approaches were tried - fill(), typed with Tab, typed with Enter, the native value setter with input and change events, the calendar picker with both dates set, and a geometry-matched filter icon - and in every case the dates appeared in the input boxes while the request still carried only paymentEventID. The date never reached the application's state. Reading the input value back does NOT prove the filter registered; capture the outgoing request instead. CORRECTION FOR THE RECORD: an automated attempt that same day reported the filter returning every row on both pages. That was the automation failing to deliver the dates, not the product. ALSO: FilterTable.countDateInputs() returns 0 for these fields, so any helper built on it silently skips the input - locate them by their YYYY-MM-DD placeholder. TC-DT-FILTER-N01 and N02 in filter-datetime-all-conditions.spec.ts are currently failing for this same automation reason rather than for an application fault. PREVIOUS NOTE, 2026-09-21, now superseded: QA 2026-09-21 BLOCKED - the Transactions grid's Date &amp; Time column filter does not filter. Measured on sub-merchant 44052730 (29,069 transactions), driving the popover directly: the date box wants YYYY-MM-DD rather than the MM/DD/YYYY the grid displays; typing 2026-09-19 lands correctly and Search does enable; but 'is equal to', 'greater than or equal to' and 'less than or equal to' each returned the full 29,069 rows, still showing 9/21 dates the filter should have excluded. Without a working date filter the comparison is a single day on one page against every transaction ever on the other, which proves nothing. SEPARATELY WORTH RAISING: Payment Stats defaults to sub-merchant 44052731 and reports card payments under it, while All Transactions lists nothing at all for that same sub-merchant; any reconciliation must pin both pages to 44052730.</t>
+          <t xml:space="preserve">QA 2026-09-24 NO LONGER BLOCKED - the Transactions Date and Time filter works. The 2026-09-21 note below it is out of date. Verified by hand on WGL over both pages: on Payments, between 2019-01-01 and 2019-12-31 returned 0 of 0 while between 2026-06-23 and 2026-09-24 returned 542; on All Transactions the same two ranges returned 0 and 903 against a 4,511 baseline. The 'between' condition did not exist on 2026-09-21 and does now, so a fix appears to have landed alongside it. RECONCILE ON THE PAYMENTS PAGE, not All Transactions: Payment Stats counts payments, while All Transactions also carries refunds and voids. Both filter correctly, so this is a choice about what is being compared rather than about which one works. STILL PIN THE SUB-MERCHANT. Payment Stats defaults to 44052731 and reports card payments under it while All Transactions lists nothing at all for that sub-merchant, so both pages must be set to 44052730 before any comparison. That half of the original note still stands. NOT YET AUTOMATED, and the reason is worth knowing before anyone tries. The Payment Stats half is straightforward. The Transactions half could not be driven from Playwright on 2026-09-24: six approaches were tried - fill(), typed with Tab, typed with Enter, the native value setter with input and change events, the calendar picker with both dates set, and a geometry-matched filter icon - and in every case the dates appeared in the input boxes while the request still carried only paymentEventID. The date never reached the application's state. Reading the input value back does NOT prove the filter registered; capture the outgoing request instead. CORRECTION FOR THE RECORD: an automated attempt that same day reported the filter returning every row on both pages. That was the automation failing to deliver the dates, not the product. ALSO: FilterTable.countDateInputs() returns 0 for these fields, so any helper built on it silently skips the input - locate them by their YYYY-MM-DD placeholder. TC-DT-FILTER-N01 and N02 in filter-datetime-all-conditions.spec.ts are currently failing for this same automation reason rather than for an application fault. PREVIOUS NOTE, 2026-09-21, now superseded: QA 2026-09-21 BLOCKED - the Transactions grid's Date &amp; Time column filter does not filter. Measured on sub-merchant 44052730 (29,069 transactions), driving the popover directly: the date box wants YYYY-MM-DD rather than the MM/DD/YYYY the grid displays; typing 2026-09-19 lands correctly and Search does enable; but 'is equal to', 'greater than or equal to' and 'less than or equal to' each returned the full 29,069 rows, still showing 9/21 dates the filter should have excluded. Without a working date filter the comparison is a single day on one page against every transaction ever on the other, which proves nothing. SEPARATELY WORTH RAISING: Payment Stats defaults to sub-merchant 44052731 and reports card payments under it, while All Transactions lists nothing at all for that same sub-merchant; any reconciliation must pin both pages to 44052730. HALF AUTOMATED 2026-09-25 - the Payment Stats side only. The Transactions side stays MANUAL and the test says so. It sets a fixed, repeatable window (the last complete calendar month) on wglUsa, sums the funding-method rows into an ACH total and a card total, checks every row carries a method and a whole-number count, and attaches the figures, the window, the per-method breakdown and the manual steps to the run so whoever finishes it has everything without re-deriving it. WHY IT IS SPLIT: the Transactions Date and Time filter WORKS - proved by hand, 2019 returned 0 of 0 and the last three months returned 542 against a 4,511 baseline. What could not be done is driving it from a test. It is a MUI X v6 DatePicker with a segmented field, and six approaches all left the date visible in the box while the request carried no filter: fill(), typed with Tab, typed with Enter, the native value setter with input and change events, typing digits into the segments, and picking from the calendar. The product is fine; the automation is not. NOTE ON THE GATEWAY: wglUsa, not ipg. IPG draws the Card Payments / ACH Payments summary directly, which would be simpler to read, but its Transactions side returns nothing (PT-NEG-12) so the manual half would have had nothing to compare against. BillPay draws the funding-method breakdown instead, hence the summing. STILL PIN THE SUB-MERCHANT before comparing: Payment Stats defaults to 44052731 while All Transactions lists nothing for it, so set both pages to 44052730. And reconcile on PAYMENTS, not All Transactions, which also carries refunds and voids.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove PS-OBS-01 from the sheet - it was an observation, not a test case
It recorded a 400 seen on page load with merchantId=undefined, which never
reproduced in automation and was marked observed-not-confirmed. Sitting in the
numbered rows it was counted as a case, so Payment Stats read as 66 of 68 when
the only real gap is PS-COL-09, which needs an India account.

The finding is not dropped - it is kept outside the sheet, with what is proven
(the endpoint is /v1/merchant/ui_config and it is called five times on a normal
load), what is not (the cause), and how to settle it: sign in through the form
rather than by injecting a token and watch the first request.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -15388,82 +15388,6 @@
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="2">
-        <v>152</v>
-      </c>
-      <c r="B153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PS-OBS-01</t>
-        </is>
-      </c>
-      <c r="C153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Payment Stats</t>
-        </is>
-      </c>
-      <c r="D153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S9. Incidental Observations</t>
-        </is>
-      </c>
-      <c r="E153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A config call fails with 400 on page load because merchantId is sent as undefined</t>
-        </is>
-      </c>
-      <c r="F153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Customer-portal user signed in through the UI (not token injection); DevTools open on the Network and Console tabs from before the first request</t>
-        </is>
-      </c>
-      <c r="G153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No fault injected. A completely healthy session.
-Gateway seen on: IPG</t>
-        </is>
-      </c>
-      <c r="H153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Open DevTools and select the Console tab, with the level filter left on Default levels
-2. Sign in to the customer portal through the sign-in form
-3. Open Payment Stats from Payment Analytics
-4. Read the console without applying any filter
-5. Switch to the Network tab and look for calls to /v1/merchant/ui_config
-6. Check the merchantId value in the query string of the first such call</t>
-        </is>
-      </c>
-      <c r="I153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Every request on a healthy page load carries a real merchant id and returns 2xx. No 400 appears in the console when nothing has gone wrong.</t>
-        </is>
-      </c>
-      <c r="J153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Medium</t>
-        </is>
-      </c>
-      <c r="M153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Automated</t>
-        </is>
-      </c>
-      <c r="O153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Observed, not confirmed</t>
-        </is>
-      </c>
-      <c r="Q153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IPG (seen); other gateways unchecked</t>
-        </is>
-      </c>
-      <c r="S153" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">QA 2026-09-24 OBSERVED, NOT YET CONFIRMED AS A DEFECT - deliberately not called a bug yet. Spotted in a merchant&amp;#8217;s own DevTools console while reproducing PS-NEG-02, on a healthy page with nothing injected: "Failed to load resource: the server responded with a status of 400" against qaapi1.tillipay.com, with merchantId=undefined in the query string. WHAT IS PROVEN: the endpoint is GET /v1/merchant/ui_config?merchantId=&lt;id&gt;, and on a normal load it is called five times over, which is worth a look on its own. WHAT IS NOT PROVEN: the cause. It does NOT reproduce in automation - on repeated IPG runs the parameter always carried a real value (526971115880) and not one request failed. The difference is that the automation writes mainMerchantId into localStorage before the app starts, so the value is ready earlier than it would be after a real sign-in. That points at a start-up ordering problem, where the first ui_config call goes out before the merchant id has been set - but that is a hypothesis, not a measurement, and it should not be written up as a defect until someone has watched it happen. TO CONFIRM: sign in through the form rather than by injecting a token, watch the Network tab from the very first request, and see whether the first ui_config call carries undefined. IMPACT IF REAL: one failed config call on every fresh sign-in, and whatever ui_config drives is left to fall back on defaults. Not blocking - the page still loads and the figures are correct.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update PS-PQ-05, PT-TIP-04 and PT-LOAD-11 status and remarks
PS-PQ-05 moves to Automated (expected fail) - the test now asserts the Expected
Result instead of the product behaviour.

PT-TIP-04 remark records that IPG is now covered as an expected failure, so the
'all gateways' scope is honest.

PT-LOAD-11 closed as not a defect and no longer needs a write-up.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -4086,7 +4086,7 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automated</t>
+          <t xml:space="preserve">Automated (expected fail)</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15 BillPay: removing every Select chip left 0 chips and the Execute button became disabled. WHY THIS SAYS Automated AND NOT Automated (expected fail), noted 2026-09-24 because the two look contradictory side by side: the test asserts what the panel does TODAY, not what it ought to do, so it passes. Emptying Select and then putting a field back frees up Group, but Having and Execute stay locked until Group itself is touched. The test records that partial recovery deliberately, so it is not mistaken for a flake. It will start FAILING the day the recovery is fixed, and that failure is the signal to flip the expectation - the failure message says so. The defect itself is written up as defect 3 in PaymentStats_Bugs.docx.</t>
+          <t xml:space="preserve">QA 2026-09-15 BillPay: removing every Select chip left 0 chips and the Execute button became disabled. WHY THIS SAYS Automated AND NOT Automated (expected fail), noted 2026-09-24 because the two look contradictory side by side: the test asserts what the panel does TODAY, not what it ought to do, so it passes. Emptying Select and then putting a field back frees up Group, but Having and Execute stay locked until Group itself is touched. The test records that partial recovery deliberately, so it is not mistaken for a flake. It will start FAILING the day the recovery is fixed, and that failure is the signal to flip the expectation - the failure message says so. The defect itself is written up as defect 3 in PaymentStats_Bugs.docx. QA 2026-09-25 REWRITTEN TO THE CASE AS WRITTEN. The test used to assert that Having STAYS disabled after a field is put back into Select - that is the product behaviour, not what this case asks for, so it passed while recording the defect. It now asserts what the Expected Result says: restoring a field re-enables Group, Having and Execute together. Marked test.fail(). Verified on 2026-09-25 - it fails on the Having assertion, which is the defect showing through. Group recovers; Having and Execute only recover once Group is touched as well, the path PS-PQ-06 covers.</t>
         </is>
       </c>
     </row>
@@ -8155,7 +8155,7 @@
       </c>
       <c r="S79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-14 SnapPay: left axis ticks read 0,5,10...60 as bare numbers - no ' k' suffix. Confirmed defect. QA 2026-09-25 STATUS CORRECTED to Automated - a test has existed for this since 2026-09-24 and the row still read Not Automated. It covers the LEFT AXIS ONLY. The right-hand axis the case also asks about never renders at all (PT-LOAD-10), so it has no ticks to judge; the test reads whatever axes do paint, so if it is ever wired up its ticks are held to the same rule without further change. The axes are found by SHAPE rather than by content, deliberately: matching on 'looks like a number' would skip the very labels this case is about, since a tick drawn as '20 k' has to be found before it can be judged. Listed as plain Automated rather than expected-fail because, like PS-PQ-05, the test asserts what the panel does today rather than what it ought to do, so it passes now and will start failing the day the suffixes are applied - and its failure message says so. Needs a write-up in the Payment Trends defects document.</t>
+          <t xml:space="preserve">QA 2026-09-14 SnapPay: left axis ticks read 0,5,10...60 as bare numbers - no &amp;#x27; k&amp;#x27; suffix. Confirmed defect. QA 2026-09-25 STATUS CORRECTED to Automated - a test has existed for this since 2026-09-24 and the row still read Not Automated. It covers the LEFT AXIS ONLY. The right-hand axis the case also asks about never renders at all (PT-LOAD-10), so it has no ticks to judge; the test reads whatever axes do paint, so if it is ever wired up its ticks are held to the same rule without further change. The axes are found by SHAPE rather than by content, deliberately: matching on &amp;#x27;looks like a number&amp;#x27; would skip the very labels this case is about, since a tick drawn as &amp;#x27;20 k&amp;#x27; has to be found before it can be judged. Listed as plain Automated rather than expected-fail because, like PS-PQ-05, the test asserts what the panel does today rather than what it ought to do, so it passes now and will start failing the day the suffixes are applied - and its failure message says so. Needs a write-up in the Payment Trends defects document. QA 2026-09-25 REVIEWED AND CLOSED - NOT A DEFECT, closed alongside PT-LOAD-10 for the same reason: unfinished configuration rather than a fault. The left axis counts PAYMENTS. If the ' k' suffix were applied, a month with 20 payments would draw a tick reading '20 k' - twenty thousand. Applying the suffix would make the chart state something false, so fixing it would be worse than leaving it. The only real effect is that a very high-volume merchant reads 50000 rather than 50 k: long, but correct. The test therefore asserts bare numbers as the CORRECT behaviour rather than as a recorded defect; the @knownissue tag has been removed and it is not marked test.fail(). NO WRITE-UP NEEDED - supersedes the earlier note asking for one in the Payment Trends defects document.</t>
         </is>
       </c>
     </row>
@@ -9654,7 +9654,7 @@
       </c>
       <c r="S94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QA 2026-09-15 SnapPay: tooltip read Token(3) and Card(52); the summary cards for the same month read Token (3) and Card (52) - identical. AUTOMATED 2026-09-25 on wglUsa, snapPay and paymentus. Measured first rather than reasoned about, by hovering and clicking the SAME bar: wglUsa Ach 43 / Card 80, snapPay Token 19 / Card 92, paymentus Ach 29 / Token 246 / Card 63 - tooltip and cards identical on all three. IPG IS DELIBERATELY EXCLUDED. There the tooltip read Ach 0 / Card 712 while the cards read Ach 0 / Card 0. That mismatch is a real defect but it is already logged twice, as PT-NEG-12 and PT-NEG-13, so running this case on IPG would fail correctly while only re-reporting those. CORRECTION to an earlier analysis: it was claimed the two numbers come from different sources and could legitimately differ, which would have made this case unsound. They agree on three of four gateways, so the case is sound and the earlier reading was wrong. Note for anyone extending it: hoverNewestMonthColumn() takes the newest bar and clickTallestBar() the tallest, so using them together compares two different months. hoverTallestBar() and pressAtPointer() were added to work on one bar.</t>
+          <t xml:space="preserve">QA 2026-09-15 SnapPay: tooltip read Token(3) and Card(52); the summary cards for the same month read Token (3) and Card (52) - identical. AUTOMATED 2026-09-25 on wglUsa, snapPay and paymentus. Measured first rather than reasoned about, by hovering and clicking the SAME bar: wglUsa Ach 43 / Card 80, snapPay Token 19 / Card 92, paymentus Ach 29 / Token 246 / Card 63 - tooltip and cards identical on all three. IPG IS DELIBERATELY EXCLUDED. There the tooltip read Ach 0 / Card 712 while the cards read Ach 0 / Card 0. That mismatch is a real defect but it is already logged twice, as PT-NEG-12 and PT-NEG-13, so running this case on IPG would fail correctly while only re-reporting those. CORRECTION to an earlier analysis: it was claimed the two numbers come from different sources and could legitimately differ, which would have made this case unsound. They agree on three of four gateways, so the case is sound and the earlier reading was wrong. Note for anyone extending it: hoverNewestMonthColumn() takes the newest bar and clickTallestBar() the tallest, so using them together compares two different months. hoverTallestBar() and pressAtPointer() were added to work on one bar. QA 2026-09-25 IPG IS NOW COVERED. The case says all gateways and the test ran only three, leaving the one gateway that disagrees out of the case. IPG has been added and marked test.fail() on its own - the other three stay unmarked so a regression in them still shows. Verified on 2026-09-25: wglUsa, snapPay and paymentus pass, ipg fails as expected. That red run is PT-NEG-12 and PT-NEG-13 showing through, already logged, not a new finding.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clear the defect wording from PT-LOAD-10 and PT-LOAD-11
Both rows still told the reader to log a defect in the Scenario and Expected
Result while the Remark said they had been reviewed and closed, so a row read
top to bottom gave contradictory instructions. The Expected Result now states
the closure and the reason; the Remarks keep the full history.
</commit_message>
<xml_diff>
--- a/PaymentAnalytics-TestCases.xlsx
+++ b/PaymentAnalytics-TestCases.xlsx
@@ -7982,7 +7982,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Right-hand value axis never renders even though one is configured (known issue)</t>
+          <t xml:space="preserve">Only the left value axis renders; the configured right-hand axis is unused</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only the left value axis is drawn; the configured right-hand axis never appears, so its fixed 0-110 domain and currency label are dead configuration (defect, log it)</t>
+          <t xml:space="preserve">Only the left value axis is drawn. The configured right-hand axis never appears, so its fixed 0-110 domain and currency label are unused configuration. REVIEWED AND CLOSED on 2026-09-25 - NOT a defect, do not log it. The amounts that axis would have carried are already one click away in the month drill-down.</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value-axis labels render as plain numbers with no ' $' or ' k' suffix (known issue)</t>
+          <t xml:space="preserve">Value-axis labels render as plain numbers with no ' $' or ' k' suffix</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -8109,7 +8109,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Both axes show bare numbers; the ' k' and ' $' suffixes never render because the label factory discards the symbol (defect, log it)</t>
+          <t xml:space="preserve">Both axes show bare numbers. The ' k' and ' $' suffixes never render because the label factory discards the symbol. REVIEWED AND CLOSED on 2026-09-25 - NOT a defect, do not log it. The left axis counts PAYMENTS, so a tick drawn as '20 k' would claim twenty thousand where there were twenty; applying the suffix would make the chart state something false.</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">

</xml_diff>